<commit_message>
Add TLE CSV input support
</commit_message>
<xml_diff>
--- a/TLE_Download/Sat_List.xlsx
+++ b/TLE_Download/Sat_List.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workspace\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workspace\TLE_Download\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DF0CEF60-1A6B-4E7B-A805-C778F80783FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9E23C0B3-2D55-4EFD-BB4D-A59E92EE24E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7336AFFB-23EE-444C-8B5E-4C0034864EFB}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="20832" windowHeight="16656" xr2:uid="{7336AFFB-23EE-444C-8B5E-4C0034864EFB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="7" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$B$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$F$21</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,6 +34,9 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
@@ -47,7 +50,25 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="68">
+  <si>
+    <t>Igor Monteiro</t>
+  </si>
+  <si>
+    <t>3538 - PU4ELT</t>
+  </si>
+  <si>
+    <t>bali</t>
+  </si>
+  <si>
+    <t>4451 - I LOVE BALI YES</t>
+  </si>
+  <si>
+    <t>Fredy Damkalis</t>
+  </si>
+  <si>
+    <t>2937 - WH6GVF UHF</t>
+  </si>
   <si>
     <t>KSM1-C</t>
   </si>
@@ -55,21 +76,45 @@
     <t>ERMIS-3</t>
   </si>
   <si>
+    <t>Jim Hutchison</t>
+  </si>
+  <si>
+    <t>3020 - Jim UHF</t>
+  </si>
+  <si>
     <t>ION SCV Astounding Alexandra</t>
   </si>
   <si>
     <t>KSM1-A</t>
   </si>
   <si>
+    <t>2026-05-06 22:19:00</t>
+  </si>
+  <si>
     <t>LUR-1</t>
   </si>
   <si>
     <t>FrontierSat</t>
   </si>
   <si>
+    <t>2026-05-06 21:49:29</t>
+  </si>
+  <si>
+    <t>342 - EA5WA Pobla Llarga</t>
+  </si>
+  <si>
     <t>SATURNIN-1</t>
   </si>
   <si>
+    <t>2026-05-06 21:28:55</t>
+  </si>
+  <si>
+    <t>Pavel Fojt</t>
+  </si>
+  <si>
+    <t>3677 - SOBE01</t>
+  </si>
+  <si>
     <t>ERNST</t>
   </si>
   <si>
@@ -79,28 +124,82 @@
     <t>ION SCV-006</t>
   </si>
   <si>
+    <t>2026-05-06 20:41:41</t>
+  </si>
+  <si>
     <t>KSM1-B</t>
   </si>
   <si>
+    <t>2026-05-06 20:24:59</t>
+  </si>
+  <si>
+    <t>2026-05-06 20:24:28</t>
+  </si>
+  <si>
+    <t>3258 - NuSpace SN1</t>
+  </si>
+  <si>
+    <t>2026-05-06 20:09:22</t>
+  </si>
+  <si>
     <t>ERMIS-2</t>
   </si>
   <si>
+    <t>2026-05-06 19:51:02</t>
+  </si>
+  <si>
     <t>CatSat</t>
   </si>
   <si>
+    <t>2026-05-06 19:29:09</t>
+  </si>
+  <si>
+    <t>1461 - VE2DSK-VHF-UHF</t>
+  </si>
+  <si>
+    <t>2026-05-06 19:24:31</t>
+  </si>
+  <si>
+    <t>2026-05-06 17:35:02</t>
+  </si>
+  <si>
+    <t>dspangler</t>
+  </si>
+  <si>
+    <t>2026-05-06 16:02:24</t>
+  </si>
+  <si>
     <t>BRO-21</t>
   </si>
   <si>
+    <t>2026-05-06 15:06:16</t>
+  </si>
+  <si>
+    <t>2026-05-06 13:58:11</t>
+  </si>
+  <si>
     <t>UND ROADS 2</t>
   </si>
   <si>
     <t>KINEIS-1A</t>
   </si>
   <si>
+    <t>2026-05-06 12:45:33</t>
+  </si>
+  <si>
     <t>ION SCV-016</t>
   </si>
   <si>
     <t>ION-MK02-SCV013</t>
+  </si>
+  <si>
+    <t>2026-05-06 03:18:08</t>
+  </si>
+  <si>
+    <t>2026-05-06 00:15:17</t>
+  </si>
+  <si>
+    <t>2026-05-05 18:46:10</t>
   </si>
   <si>
     <t>NORAD ID</t>
@@ -111,7 +210,53 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
+    <t>2026-05-05 15:17:29</t>
+  </si>
+  <si>
     <t>KSM1-D</t>
+  </si>
+  <si>
+    <t>2026-05-04 23:54:53</t>
+  </si>
+  <si>
+    <t>   6</t>
+  </si>
+  <si>
+    <t>   3</t>
+  </si>
+  <si>
+    <t>   2</t>
+  </si>
+  <si>
+    <t>   1</t>
+  </si>
+  <si>
+    <t>   11</t>
+  </si>
+  <si>
+    <t>   89</t>
+  </si>
+  <si>
+    <t>   188</t>
+  </si>
+  <si>
+    <t>   16</t>
+  </si>
+  <si>
+    <t>Timeframe</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Results</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Observer</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Station</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>SAT_Name</t>
@@ -250,7 +395,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -260,7 +405,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -269,13 +414,16 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -285,7 +433,7 @@
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="10">
     <dxf>
       <font>
         <b val="0"/>
@@ -365,6 +513,174 @@
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <color auto="1"/>
+        <name val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="major"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <color auto="1"/>
+        <name val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="major"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <color auto="1"/>
+        <name val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="major"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <color auto="1"/>
+        <name val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="major"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
       <border outline="0">
         <top style="thin">
           <color indexed="64"/>
@@ -444,9 +760,13 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{37F316E7-41DB-4B1F-85A8-120B29DBD80F}" name="표8" displayName="표8" ref="A1:B21" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3" totalsRowBorderDxfId="2">
-  <tableColumns count="2">
-    <tableColumn id="2" xr3:uid="{EFDA5C7B-E709-4C5A-831B-BC31841EA2F4}" name="Satellite" dataDxfId="1"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{37F316E7-41DB-4B1F-85A8-120B29DBD80F}" name="표8" displayName="표8" ref="A1:F21" totalsRowShown="0" headerRowDxfId="9" headerRowBorderDxfId="8" tableBorderDxfId="7" totalsRowBorderDxfId="6">
+  <tableColumns count="6">
+    <tableColumn id="2" xr3:uid="{EFDA5C7B-E709-4C5A-831B-BC31841EA2F4}" name="SAT_Name" dataDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{7D46265B-691B-48F8-AE55-779CA174089C}" name="Timeframe" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{AD6FFAA2-BA7E-48ED-92C2-2D633CB898C2}" name="Results" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{332193FC-FB8A-4911-8226-C8C2140B4E33}" name="Observer" dataDxfId="2"/>
+    <tableColumn id="8" xr3:uid="{78F39428-398F-4213-89F2-9826DA7B40AC}" name="Station" dataDxfId="1"/>
     <tableColumn id="9" xr3:uid="{2830342C-8A2C-4B7A-B14E-3CE6B69DCCDC}" name="NORAD ID" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -770,337 +1090,791 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F24BE7C-2308-4666-8E39-AD50BFED458C}">
-  <dimension ref="A1:C73"/>
+  <dimension ref="A1:F73"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999"/>
   <cols>
     <col min="1" max="1" width="24" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.8984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="100.59765625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15" style="2" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="10.5" style="2" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="11.69921875" style="2" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="20" style="2" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="12.8984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="100.59765625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="6" customFormat="1" ht="15.6">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:6" s="7" customFormat="1" ht="15.6">
+      <c r="A1" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" s="5">
+        <v>60246</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F3" s="5">
+        <v>68468</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F4" s="5">
+        <v>68420</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B5" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="F5" s="5">
+        <v>60528</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F6" s="6">
+        <v>69015</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F7" s="6">
+        <v>68435</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F8" s="5">
+        <v>52761</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F9" s="5">
+        <v>60573</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F10" s="5">
+        <v>62628</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F11" s="5">
+        <v>58300</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F12" s="5">
+        <v>60084</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="17.399999999999999" customHeight="1">
+      <c r="A13" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F13" s="5">
+        <v>46912</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F14" s="5">
+        <v>46914</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="17.399999999999999" customHeight="1">
+      <c r="A15" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F15" s="4">
+        <v>46906</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F16" s="5">
+        <v>46907</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
+      <c r="A17" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F17" s="5">
+        <v>60506</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="17.399999999999999" customHeight="1">
+      <c r="A18" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F18" s="5">
+        <v>64549</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="17.399999999999999" customHeight="1">
+      <c r="A19" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F19" s="6">
+        <v>98311</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6">
+      <c r="A20" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F20" s="6">
+        <v>98367</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6">
+      <c r="A21" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B21" s="3" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B2" s="5">
-        <v>60246</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2">
-      <c r="A3" s="3" t="s">
+      <c r="C21" s="3"/>
+      <c r="D21" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="B3" s="5">
-        <v>68468</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2">
-      <c r="A4" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" s="5">
-        <v>68420</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2">
-      <c r="A5" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" s="5">
-        <v>60528</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2">
-      <c r="A6" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6" s="3">
-        <v>69015</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2">
-      <c r="A7" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="B7" s="3">
-        <v>68435</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2">
-      <c r="A8" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" s="5">
-        <v>52761</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2">
-      <c r="A9" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B9" s="5">
-        <v>60573</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2">
-      <c r="A10" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10" s="5">
-        <v>62628</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2">
-      <c r="A11" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B11" s="5">
-        <v>58300</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2">
-      <c r="A12" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B12" s="5">
-        <v>60084</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" ht="17.399999999999999" customHeight="1">
-      <c r="A13" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B13" s="5">
-        <v>46912</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2">
-      <c r="A14" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B14" s="5">
-        <v>46914</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" ht="17.399999999999999" customHeight="1">
-      <c r="A15" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B15" s="4">
-        <v>46906</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2">
-      <c r="A16" s="3" t="s">
+      <c r="E21" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="5">
-        <v>46907</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2">
-      <c r="A17" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B17" s="5">
-        <v>60506</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="17.399999999999999" customHeight="1">
-      <c r="A18" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B18" s="5">
-        <v>64549</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" ht="17.399999999999999" customHeight="1">
-      <c r="A19" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B19" s="3">
-        <v>98311</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2">
-      <c r="A20" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B20" s="3">
-        <v>98367</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2">
-      <c r="A21" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="B21" s="9">
+      <c r="F21" s="10">
         <v>98671</v>
       </c>
     </row>
-    <row r="22" spans="1:2">
+    <row r="22" spans="1:6">
       <c r="A22"/>
-    </row>
-    <row r="23" spans="1:2">
+      <c r="B22"/>
+      <c r="C22"/>
+      <c r="D22"/>
+      <c r="E22"/>
+    </row>
+    <row r="23" spans="1:6">
       <c r="A23"/>
-    </row>
-    <row r="24" spans="1:2">
+      <c r="B23"/>
+      <c r="C23"/>
+      <c r="D23"/>
+      <c r="E23"/>
+    </row>
+    <row r="24" spans="1:6">
       <c r="A24"/>
-    </row>
-    <row r="25" spans="1:2">
+      <c r="B24"/>
+      <c r="C24"/>
+      <c r="D24"/>
+      <c r="E24"/>
+    </row>
+    <row r="25" spans="1:6">
       <c r="A25"/>
-    </row>
-    <row r="26" spans="1:2">
+      <c r="B25"/>
+      <c r="C25"/>
+      <c r="D25"/>
+      <c r="E25"/>
+    </row>
+    <row r="26" spans="1:6">
       <c r="A26"/>
-    </row>
-    <row r="27" spans="1:2">
+      <c r="B26"/>
+      <c r="C26"/>
+      <c r="D26"/>
+      <c r="E26"/>
+    </row>
+    <row r="27" spans="1:6">
       <c r="A27"/>
-    </row>
-    <row r="28" spans="1:2">
+      <c r="B27"/>
+      <c r="C27"/>
+      <c r="D27"/>
+      <c r="E27"/>
+    </row>
+    <row r="28" spans="1:6">
       <c r="A28"/>
-    </row>
-    <row r="29" spans="1:2">
+      <c r="B28"/>
+      <c r="C28"/>
+      <c r="D28"/>
+      <c r="E28"/>
+    </row>
+    <row r="29" spans="1:6">
       <c r="A29"/>
-    </row>
-    <row r="30" spans="1:2">
+      <c r="B29"/>
+      <c r="C29"/>
+      <c r="D29"/>
+      <c r="E29"/>
+    </row>
+    <row r="30" spans="1:6">
       <c r="A30"/>
-    </row>
-    <row r="31" spans="1:2">
+      <c r="B30"/>
+      <c r="C30"/>
+      <c r="D30"/>
+      <c r="E30"/>
+    </row>
+    <row r="31" spans="1:6">
       <c r="A31"/>
-    </row>
-    <row r="32" spans="1:2">
+      <c r="B31"/>
+      <c r="C31"/>
+      <c r="D31"/>
+      <c r="E31"/>
+    </row>
+    <row r="32" spans="1:6">
       <c r="A32"/>
-    </row>
-    <row r="33" spans="1:1">
+      <c r="B32"/>
+      <c r="C32"/>
+      <c r="D32"/>
+      <c r="E32"/>
+    </row>
+    <row r="33" spans="1:5">
       <c r="A33"/>
-    </row>
-    <row r="34" spans="1:1">
+      <c r="B33"/>
+      <c r="C33"/>
+      <c r="D33"/>
+      <c r="E33"/>
+    </row>
+    <row r="34" spans="1:5">
       <c r="A34"/>
-    </row>
-    <row r="35" spans="1:1">
+      <c r="B34"/>
+      <c r="C34"/>
+      <c r="D34"/>
+      <c r="E34"/>
+    </row>
+    <row r="35" spans="1:5">
       <c r="A35"/>
-    </row>
-    <row r="36" spans="1:1">
+      <c r="B35"/>
+      <c r="C35"/>
+      <c r="D35"/>
+      <c r="E35"/>
+    </row>
+    <row r="36" spans="1:5">
       <c r="A36"/>
-    </row>
-    <row r="37" spans="1:1">
+      <c r="B36"/>
+      <c r="C36"/>
+      <c r="D36"/>
+      <c r="E36"/>
+    </row>
+    <row r="37" spans="1:5">
       <c r="A37"/>
-    </row>
-    <row r="38" spans="1:1">
+      <c r="B37"/>
+      <c r="C37"/>
+      <c r="D37"/>
+      <c r="E37"/>
+    </row>
+    <row r="38" spans="1:5">
       <c r="A38"/>
-    </row>
-    <row r="39" spans="1:1">
+      <c r="B38"/>
+      <c r="C38"/>
+      <c r="D38"/>
+      <c r="E38"/>
+    </row>
+    <row r="39" spans="1:5">
       <c r="A39"/>
-    </row>
-    <row r="40" spans="1:1">
+      <c r="B39"/>
+      <c r="C39"/>
+      <c r="D39"/>
+      <c r="E39"/>
+    </row>
+    <row r="40" spans="1:5">
       <c r="A40"/>
-    </row>
-    <row r="41" spans="1:1">
+      <c r="B40"/>
+      <c r="C40"/>
+      <c r="D40"/>
+      <c r="E40"/>
+    </row>
+    <row r="41" spans="1:5">
       <c r="A41"/>
-    </row>
-    <row r="42" spans="1:1">
+      <c r="B41"/>
+      <c r="C41"/>
+      <c r="D41"/>
+      <c r="E41"/>
+    </row>
+    <row r="42" spans="1:5">
       <c r="A42"/>
-    </row>
-    <row r="43" spans="1:1">
+      <c r="B42"/>
+      <c r="C42"/>
+      <c r="D42"/>
+      <c r="E42"/>
+    </row>
+    <row r="43" spans="1:5">
       <c r="A43"/>
-    </row>
-    <row r="44" spans="1:1">
+      <c r="B43"/>
+      <c r="C43"/>
+      <c r="D43"/>
+      <c r="E43"/>
+    </row>
+    <row r="44" spans="1:5">
       <c r="A44"/>
-    </row>
-    <row r="45" spans="1:1">
+      <c r="B44"/>
+      <c r="C44"/>
+      <c r="D44"/>
+      <c r="E44"/>
+    </row>
+    <row r="45" spans="1:5">
       <c r="A45"/>
-    </row>
-    <row r="46" spans="1:1">
+      <c r="B45"/>
+      <c r="C45"/>
+      <c r="D45"/>
+      <c r="E45"/>
+    </row>
+    <row r="46" spans="1:5">
       <c r="A46"/>
-    </row>
-    <row r="47" spans="1:1">
+      <c r="B46"/>
+      <c r="C46"/>
+      <c r="D46"/>
+      <c r="E46"/>
+    </row>
+    <row r="47" spans="1:5">
       <c r="A47"/>
-    </row>
-    <row r="48" spans="1:1">
+      <c r="B47"/>
+      <c r="C47"/>
+      <c r="D47"/>
+      <c r="E47"/>
+    </row>
+    <row r="48" spans="1:5">
       <c r="A48"/>
-    </row>
-    <row r="49" spans="1:1">
+      <c r="B48"/>
+      <c r="C48"/>
+      <c r="D48"/>
+      <c r="E48"/>
+    </row>
+    <row r="49" spans="1:5">
       <c r="A49"/>
-    </row>
-    <row r="50" spans="1:1">
+      <c r="B49"/>
+      <c r="C49"/>
+      <c r="D49"/>
+      <c r="E49"/>
+    </row>
+    <row r="50" spans="1:5">
       <c r="A50"/>
-    </row>
-    <row r="51" spans="1:1">
+      <c r="B50"/>
+      <c r="C50"/>
+      <c r="D50"/>
+      <c r="E50"/>
+    </row>
+    <row r="51" spans="1:5">
       <c r="A51"/>
-    </row>
-    <row r="52" spans="1:1">
+      <c r="B51"/>
+      <c r="C51"/>
+      <c r="D51"/>
+      <c r="E51"/>
+    </row>
+    <row r="52" spans="1:5">
       <c r="A52"/>
-    </row>
-    <row r="53" spans="1:1">
+      <c r="B52"/>
+      <c r="C52"/>
+      <c r="D52"/>
+      <c r="E52"/>
+    </row>
+    <row r="53" spans="1:5">
       <c r="A53"/>
-    </row>
-    <row r="54" spans="1:1">
+      <c r="B53"/>
+      <c r="C53"/>
+      <c r="D53"/>
+      <c r="E53"/>
+    </row>
+    <row r="54" spans="1:5">
       <c r="A54"/>
-    </row>
-    <row r="55" spans="1:1">
+      <c r="B54"/>
+      <c r="C54"/>
+      <c r="D54"/>
+      <c r="E54"/>
+    </row>
+    <row r="55" spans="1:5">
       <c r="A55"/>
-    </row>
-    <row r="56" spans="1:1">
+      <c r="B55"/>
+      <c r="C55"/>
+      <c r="D55"/>
+      <c r="E55"/>
+    </row>
+    <row r="56" spans="1:5">
       <c r="A56"/>
-    </row>
-    <row r="57" spans="1:1">
+      <c r="B56"/>
+      <c r="C56"/>
+      <c r="D56"/>
+      <c r="E56"/>
+    </row>
+    <row r="57" spans="1:5">
       <c r="A57"/>
-    </row>
-    <row r="58" spans="1:1">
+      <c r="B57"/>
+      <c r="C57"/>
+      <c r="D57"/>
+      <c r="E57"/>
+    </row>
+    <row r="58" spans="1:5">
       <c r="A58"/>
-    </row>
-    <row r="59" spans="1:1">
+      <c r="B58"/>
+      <c r="C58"/>
+      <c r="D58"/>
+      <c r="E58"/>
+    </row>
+    <row r="59" spans="1:5">
       <c r="A59"/>
-    </row>
-    <row r="60" spans="1:1">
+      <c r="B59"/>
+      <c r="C59"/>
+      <c r="D59"/>
+      <c r="E59"/>
+    </row>
+    <row r="60" spans="1:5">
       <c r="A60"/>
-    </row>
-    <row r="61" spans="1:1">
+      <c r="B60"/>
+      <c r="C60"/>
+      <c r="D60"/>
+      <c r="E60"/>
+    </row>
+    <row r="61" spans="1:5">
       <c r="A61"/>
-    </row>
-    <row r="62" spans="1:1">
+      <c r="B61"/>
+      <c r="C61"/>
+      <c r="D61"/>
+      <c r="E61"/>
+    </row>
+    <row r="62" spans="1:5">
       <c r="A62"/>
-    </row>
-    <row r="63" spans="1:1">
+      <c r="B62"/>
+      <c r="C62"/>
+      <c r="D62"/>
+      <c r="E62"/>
+    </row>
+    <row r="63" spans="1:5">
       <c r="A63"/>
-    </row>
-    <row r="64" spans="1:1">
+      <c r="B63"/>
+      <c r="C63"/>
+      <c r="D63"/>
+      <c r="E63"/>
+    </row>
+    <row r="64" spans="1:5">
       <c r="A64"/>
-    </row>
-    <row r="65" spans="1:1">
+      <c r="B64"/>
+      <c r="C64"/>
+      <c r="D64"/>
+      <c r="E64"/>
+    </row>
+    <row r="65" spans="1:5">
       <c r="A65"/>
-    </row>
-    <row r="66" spans="1:1">
+      <c r="B65"/>
+      <c r="C65"/>
+      <c r="D65"/>
+      <c r="E65"/>
+    </row>
+    <row r="66" spans="1:5">
       <c r="A66"/>
-    </row>
-    <row r="67" spans="1:1">
+      <c r="B66"/>
+      <c r="C66"/>
+      <c r="D66"/>
+      <c r="E66"/>
+    </row>
+    <row r="67" spans="1:5">
       <c r="A67"/>
-    </row>
-    <row r="68" spans="1:1">
+      <c r="B67"/>
+      <c r="C67"/>
+      <c r="D67"/>
+      <c r="E67"/>
+    </row>
+    <row r="68" spans="1:5">
       <c r="A68"/>
-    </row>
-    <row r="69" spans="1:1">
+      <c r="B68"/>
+      <c r="C68"/>
+      <c r="D68"/>
+      <c r="E68"/>
+    </row>
+    <row r="69" spans="1:5">
       <c r="A69"/>
-    </row>
-    <row r="70" spans="1:1">
+      <c r="B69"/>
+      <c r="C69"/>
+      <c r="D69"/>
+      <c r="E69"/>
+    </row>
+    <row r="70" spans="1:5">
       <c r="A70"/>
-    </row>
-    <row r="71" spans="1:1">
+      <c r="B70"/>
+      <c r="C70"/>
+      <c r="D70"/>
+      <c r="E70"/>
+    </row>
+    <row r="71" spans="1:5">
       <c r="A71"/>
-    </row>
-    <row r="72" spans="1:1">
+      <c r="B71"/>
+      <c r="C71"/>
+      <c r="D71"/>
+      <c r="E71"/>
+    </row>
+    <row r="72" spans="1:5">
       <c r="A72"/>
-    </row>
-    <row r="73" spans="1:1">
+      <c r="B72"/>
+      <c r="C72"/>
+      <c r="D72"/>
+      <c r="E72"/>
+    </row>
+    <row r="73" spans="1:5">
       <c r="A73"/>
+      <c r="B73"/>
+      <c r="C73"/>
+      <c r="D73"/>
+      <c r="E73"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>